<commit_message>
timeout and expected url not matching fix
</commit_message>
<xml_diff>
--- a/reports/Website_Link_Report.xlsx
+++ b/reports/Website_Link_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="64">
   <si>
     <t>Website Link Validation Report</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2/8/2026</t>
+    <t>4/8/2026</t>
   </si>
   <si>
     <t>Browser</t>
@@ -40,7 +40,7 @@
     <t>Execution Time</t>
   </si>
   <si>
-    <t>30.70 sec</t>
+    <t>30.18 sec</t>
   </si>
   <si>
     <t>Summary</t>
@@ -112,33 +112,6 @@
     <t>Accessibility Menu</t>
   </si>
   <si>
-    <t>Banners</t>
-  </si>
-  <si>
-    <t>locator('.slick-slide.slick-current.slick-active').locator('.subtitle') Banner</t>
-  </si>
-  <si>
-    <t>Banner locator('.slick-slide.slick-current.slick-active').locator('.subtitle') is visible</t>
-  </si>
-  <si>
-    <t>locator('.slick-slide.slick-current.slick-active').locator('h2') Banner</t>
-  </si>
-  <si>
-    <t>Banner locator('.slick-slide.slick-current.slick-active').locator('h2') is visible</t>
-  </si>
-  <si>
-    <t>locator('.slick-slide.slick-current.slick-active').locator('.txt') Banner</t>
-  </si>
-  <si>
-    <t>Banner locator('.slick-slide.slick-current.slick-active').locator('.txt') is visible</t>
-  </si>
-  <si>
-    <t>locator('.slick-slide.slick-current.slick-active').locator('.btn.btn--orange') Banner</t>
-  </si>
-  <si>
-    <t>Banner locator('.slick-slide.slick-current.slick-active').locator('.btn.btn--orange') is visible</t>
-  </si>
-  <si>
     <t>Info Card</t>
   </si>
   <si>
@@ -172,7 +145,7 @@
     <t>More info</t>
   </si>
   <si>
-    <t>Successfully Navigated to This month at the Alimentarium page</t>
+    <t>Successfully navigated to "This month at the Alimentarium" page</t>
   </si>
   <si>
     <t>School activities</t>
@@ -181,7 +154,7 @@
     <t>Info Card School activities is visible</t>
   </si>
   <si>
-    <t>Successfully Navigated to School activities page</t>
+    <t>Successfully navigated to "School activities" page</t>
   </si>
   <si>
     <t>Systema Alimentarium</t>
@@ -208,7 +181,28 @@
     <t>Find out more</t>
   </si>
   <si>
-    <t>Successfully Navigated to Systema Alimentarium page</t>
+    <t>Successfully navigated to "Systema Alimentarium" page</t>
+  </si>
+  <si>
+    <t>Garden</t>
+  </si>
+  <si>
+    <t>Info Card Garden is visible</t>
+  </si>
+  <si>
+    <t>See more button</t>
+  </si>
+  <si>
+    <t>See more Button is visible</t>
+  </si>
+  <si>
+    <t>Click on See more</t>
+  </si>
+  <si>
+    <t>See more</t>
+  </si>
+  <si>
+    <t>Successfully navigated to "Garden" page</t>
   </si>
 </sst>
 </file>
@@ -888,16 +882,16 @@
         <v>11</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -905,16 +899,16 @@
         <v>12</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -922,16 +916,16 @@
         <v>13</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -939,16 +933,16 @@
         <v>14</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -956,16 +950,16 @@
         <v>15</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -973,16 +967,16 @@
         <v>16</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -990,16 +984,16 @@
         <v>17</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1007,16 +1001,16 @@
         <v>18</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1024,16 +1018,16 @@
         <v>19</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1041,16 +1035,16 @@
         <v>20</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1058,10 +1052,10 @@
         <v>21</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>22</v>
@@ -1075,7 +1069,7 @@
         <v>22</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>57</v>
@@ -1092,16 +1086,16 @@
         <v>23</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1109,16 +1103,16 @@
         <v>24</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1126,16 +1120,16 @@
         <v>25</v>
       </c>
       <c r="B42" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E42" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Banner Navigation and timeout issue
</commit_message>
<xml_diff>
--- a/reports/Website_Link_Report.xlsx
+++ b/reports/Website_Link_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="73">
   <si>
     <t>Website Link Validation Report</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>4/8/2026</t>
+    <t>5/8/2026</t>
   </si>
   <si>
     <t>Browser</t>
@@ -40,7 +40,7 @@
     <t>Execution Time</t>
   </si>
   <si>
-    <t>30.18 sec</t>
+    <t>70.60 sec</t>
   </si>
   <si>
     <t>Summary</t>
@@ -112,6 +112,33 @@
     <t>Accessibility Menu</t>
   </si>
   <si>
+    <t>Banner</t>
+  </si>
+  <si>
+    <t>Swiss Museum Prize 2026</t>
+  </si>
+  <si>
+    <t>Banner verified</t>
+  </si>
+  <si>
+    <t>Banner Navigation</t>
+  </si>
+  <si>
+    <t>Successfully navigated</t>
+  </si>
+  <si>
+    <t>Share your story</t>
+  </si>
+  <si>
+    <t>“Alima”</t>
+  </si>
+  <si>
+    <t>Cooking together</t>
+  </si>
+  <si>
+    <t>Open kitchen</t>
+  </si>
+  <si>
     <t>Info Card</t>
   </si>
   <si>
@@ -139,6 +166,42 @@
     <t>More info Button is visible</t>
   </si>
   <si>
+    <t>School activities</t>
+  </si>
+  <si>
+    <t>Info Card School activities is visible</t>
+  </si>
+  <si>
+    <t>Systema Alimentarium</t>
+  </si>
+  <si>
+    <t>Info Card Systema Alimentarium is visible</t>
+  </si>
+  <si>
+    <t>Exhibition</t>
+  </si>
+  <si>
+    <t>Exhibition header is visible</t>
+  </si>
+  <si>
+    <t>Find out more button</t>
+  </si>
+  <si>
+    <t>Find out more Button is visible</t>
+  </si>
+  <si>
+    <t>Garden</t>
+  </si>
+  <si>
+    <t>Info Card Garden is visible</t>
+  </si>
+  <si>
+    <t>See more button</t>
+  </si>
+  <si>
+    <t>See more Button is visible</t>
+  </si>
+  <si>
     <t>Click on More info</t>
   </si>
   <si>
@@ -148,33 +211,9 @@
     <t>Successfully navigated to "This month at the Alimentarium" page</t>
   </si>
   <si>
-    <t>School activities</t>
-  </si>
-  <si>
-    <t>Info Card School activities is visible</t>
-  </si>
-  <si>
     <t>Successfully navigated to "School activities" page</t>
   </si>
   <si>
-    <t>Systema Alimentarium</t>
-  </si>
-  <si>
-    <t>Info Card Systema Alimentarium is visible</t>
-  </si>
-  <si>
-    <t>Exhibition</t>
-  </si>
-  <si>
-    <t>Exhibition header is visible</t>
-  </si>
-  <si>
-    <t>Find out more button</t>
-  </si>
-  <si>
-    <t>Find out more Button is visible</t>
-  </si>
-  <si>
     <t>Click on Find out more</t>
   </si>
   <si>
@@ -182,18 +221,6 @@
   </si>
   <si>
     <t>Successfully navigated to "Systema Alimentarium" page</t>
-  </si>
-  <si>
-    <t>Garden</t>
-  </si>
-  <si>
-    <t>Info Card Garden is visible</t>
-  </si>
-  <si>
-    <t>See more button</t>
-  </si>
-  <si>
-    <t>See more Button is visible</t>
   </si>
   <si>
     <t>Click on See more</t>
@@ -606,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="30" customWidth="1"/>
@@ -676,10 +703,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B13">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -885,13 +912,13 @@
         <v>36</v>
       </c>
       <c r="C28" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -899,16 +926,16 @@
         <v>12</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -916,16 +943,16 @@
         <v>13</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -936,13 +963,13 @@
         <v>33</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -953,13 +980,13 @@
         <v>36</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -967,7 +994,7 @@
         <v>16</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>40</v>
@@ -976,7 +1003,7 @@
         <v>22</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -984,16 +1011,16 @@
         <v>17</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1004,13 +1031,13 @@
         <v>33</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1021,13 +1048,13 @@
         <v>36</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1035,16 +1062,16 @@
         <v>20</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1052,16 +1079,16 @@
         <v>21</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1069,16 +1096,16 @@
         <v>22</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1086,16 +1113,16 @@
         <v>23</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1103,16 +1130,16 @@
         <v>24</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1120,16 +1147,186 @@
         <v>25</v>
       </c>
       <c r="B42" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="4">
+        <v>26</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>27</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>28</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>29</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>30</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>31</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C48" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="D48" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D42" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E42" s="4" t="s">
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>32</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>63</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>33</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>34</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>35</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added separate for each components
</commit_message>
<xml_diff>
--- a/reports/Website_Link_Report.xlsx
+++ b/reports/Website_Link_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="69">
   <si>
     <t>Website Link Validation Report</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>5/8/2026</t>
+    <t>6/8/2026</t>
   </si>
   <si>
     <t>Browser</t>
@@ -40,7 +40,7 @@
     <t>Execution Time</t>
   </si>
   <si>
-    <t>70.60 sec</t>
+    <t>78.31 sec</t>
   </si>
   <si>
     <t>Summary</t>
@@ -73,18 +73,66 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>Banner</t>
+  </si>
+  <si>
+    <t>Competition</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Text verified</t>
+  </si>
+  <si>
+    <t>Swiss Museum Prize 2026</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Visible</t>
+  </si>
+  <si>
+    <t>More info</t>
+  </si>
+  <si>
+    <t>Banner Navigation</t>
+  </si>
+  <si>
+    <t>Successfully navigated</t>
+  </si>
+  <si>
+    <t>Testimonies</t>
+  </si>
+  <si>
+    <t>Share your story</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>“Alima”</t>
+  </si>
+  <si>
+    <t>Workshops</t>
+  </si>
+  <si>
+    <t>Cooking together</t>
+  </si>
+  <si>
+    <t>Animation</t>
+  </si>
+  <si>
+    <t>Open kitchen</t>
+  </si>
+  <si>
     <t>Header</t>
   </si>
   <si>
     <t>Logo</t>
   </si>
   <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>Visible</t>
-  </si>
-  <si>
     <t>Search Icon</t>
   </si>
   <si>
@@ -100,9 +148,6 @@
     <t>Visit Menu</t>
   </si>
   <si>
-    <t>Menu is visible</t>
-  </si>
-  <si>
     <t>Learn &amp; Play Menu</t>
   </si>
   <si>
@@ -112,100 +157,43 @@
     <t>Accessibility Menu</t>
   </si>
   <si>
-    <t>Banner</t>
-  </si>
-  <si>
-    <t>Swiss Museum Prize 2026</t>
-  </si>
-  <si>
-    <t>Banner verified</t>
-  </si>
-  <si>
-    <t>Banner Navigation</t>
-  </si>
-  <si>
-    <t>Successfully navigated</t>
-  </si>
-  <si>
-    <t>Share your story</t>
-  </si>
-  <si>
-    <t>“Alima”</t>
-  </si>
-  <si>
-    <t>Cooking together</t>
-  </si>
-  <si>
-    <t>Open kitchen</t>
-  </si>
-  <si>
     <t>Info Card</t>
   </si>
   <si>
     <t>This month at the Alimentarium</t>
   </si>
   <si>
-    <t>Info Card This month at the Alimentarium is visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Info Card Header/label </t>
+    <t>Info Card Header/label</t>
   </si>
   <si>
     <t>Activities</t>
   </si>
   <si>
-    <t>Activities header is visible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Info Card More info button </t>
+    <t>Info Card More info button</t>
   </si>
   <si>
     <t>More info button</t>
   </si>
   <si>
-    <t>More info Button is visible</t>
-  </si>
-  <si>
     <t>School activities</t>
   </si>
   <si>
-    <t>Info Card School activities is visible</t>
-  </si>
-  <si>
     <t>Systema Alimentarium</t>
   </si>
   <si>
-    <t>Info Card Systema Alimentarium is visible</t>
-  </si>
-  <si>
     <t>Exhibition</t>
   </si>
   <si>
-    <t>Exhibition header is visible</t>
-  </si>
-  <si>
     <t>Find out more button</t>
   </si>
   <si>
-    <t>Find out more Button is visible</t>
-  </si>
-  <si>
     <t>Garden</t>
   </si>
   <si>
-    <t>Info Card Garden is visible</t>
-  </si>
-  <si>
     <t>See more button</t>
   </si>
   <si>
-    <t>See more Button is visible</t>
-  </si>
-  <si>
     <t>Click on More info</t>
-  </si>
-  <si>
-    <t>More info</t>
   </si>
   <si>
     <t>Successfully navigated to "This month at the Alimentarium" page</t>
@@ -633,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="30" customWidth="1"/>
@@ -703,10 +691,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="B13">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -782,7 +770,7 @@
         <v>22</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -793,7 +781,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>22</v>
@@ -807,16 +795,16 @@
         <v>5</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -827,13 +815,13 @@
         <v>20</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -844,13 +832,13 @@
         <v>20</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -861,13 +849,13 @@
         <v>20</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -878,13 +866,13 @@
         <v>20</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -892,16 +880,16 @@
         <v>10</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -909,16 +897,16 @@
         <v>11</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -926,16 +914,16 @@
         <v>12</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="D29" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -943,16 +931,16 @@
         <v>13</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -960,16 +948,16 @@
         <v>14</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -977,16 +965,16 @@
         <v>15</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -994,16 +982,16 @@
         <v>16</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1011,16 +999,16 @@
         <v>17</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1028,16 +1016,16 @@
         <v>18</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1045,16 +1033,16 @@
         <v>19</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1062,16 +1050,16 @@
         <v>20</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1079,16 +1067,16 @@
         <v>21</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1096,16 +1084,16 @@
         <v>22</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1113,16 +1101,16 @@
         <v>23</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1130,16 +1118,16 @@
         <v>24</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1147,16 +1135,16 @@
         <v>25</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1164,16 +1152,16 @@
         <v>26</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1181,16 +1169,16 @@
         <v>27</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1198,16 +1186,16 @@
         <v>28</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>58</v>
+        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1215,16 +1203,16 @@
         <v>29</v>
       </c>
       <c r="B46" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C46" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C46" s="4" t="s">
-        <v>59</v>
-      </c>
       <c r="D46" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -1232,16 +1220,16 @@
         <v>30</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1249,16 +1237,16 @@
         <v>31</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -1266,16 +1254,16 @@
         <v>32</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>65</v>
+        <v>26</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -1283,16 +1271,16 @@
         <v>33</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -1300,16 +1288,16 @@
         <v>34</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -1317,16 +1305,271 @@
         <v>35</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>72</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>36</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>37</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>38</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>39</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>40</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>41</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>42</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>43</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>44</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>45</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>46</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>47</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>48</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>49</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>50</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>